<commit_message>
Update data config for Coding VF5NP
</commit_message>
<xml_diff>
--- a/config/Coding/VF5NP_ACM_F108.xlsx
+++ b/config/Coding/VF5NP_ACM_F108.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\REDO\CODINGTOOL\config\Coding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5DEC9D-1B4F-4AE3-8BB8-61024D0C4FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C52D6DA-1E25-412C-902A-82E07B162805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23232" windowHeight="12432" xr2:uid="{ABFBD026-99C8-4534-880F-EF7C8CBF5F13}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{ABFBD026-99C8-4534-880F-EF7C8CBF5F13}"/>
   </bookViews>
   <sheets>
     <sheet name="CDS Coding" sheetId="1" r:id="rId1"/>

</xml_diff>